<commit_message>
add: --Backups --Test Fixed: --massage.xlsx
</commit_message>
<xml_diff>
--- a/Bot/misc/categories/massage.xlsx
+++ b/Bot/misc/categories/massage.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\ВАЖНОЕ\rynoksmm rebuild\Bot\misc\categories\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -21,12 +21,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="22">
   <si>
-    <t>Категория массажа</t>
-  </si>
-  <si>
-    <t>Тип массажа</t>
-  </si>
-  <si>
     <t>Лечебный массаж</t>
   </si>
   <si>
@@ -85,6 +79,12 @@
   </si>
   <si>
     <t>ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Категория </t>
+  </si>
+  <si>
+    <t>Название</t>
   </si>
 </sst>
 </file>
@@ -455,19 +455,19 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="41.140625" customWidth="1"/>
-    <col min="3" max="3" width="37.28515625" customWidth="1"/>
+    <col min="2" max="2" width="37.28515625" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -475,10 +475,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -486,10 +486,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -497,10 +497,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -508,10 +508,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -519,10 +519,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -530,10 +530,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -541,10 +541,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -552,10 +552,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -563,10 +563,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -574,10 +574,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -585,10 +585,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -596,10 +596,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -607,10 +607,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -618,10 +618,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -629,10 +629,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>